<commit_message>
feat: convert counted units to store packs before the cart (#382)
- optional units_per_pack column: the cart run buys ceil(units needed / units per pack), 0 when nothing is needed, units unchanged when unset
- applied once where the cart run reads the inventory, with one info line per converted item
- item sheet and Add item form carry the field; PUT keeps it when omitted and clears it on null
- "buy" reads units and packs (14 units -> 3 packs) in the Items, Audit and Shop lists
- docs/items.md explains the field; the example sheet gains the column
</commit_message>
<xml_diff>
--- a/data/list.example.xlsx
+++ b/data/list.example.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,43 +413,48 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>super</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>buscador</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>lugar</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>comida</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>cantidad</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>tenemos</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>comprar</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>units_per_pack</t>
         </is>
       </c>
     </row>
@@ -491,6 +484,7 @@
       <c r="G2" t="n">
         <v>1</v>
       </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -518,6 +512,7 @@
       <c r="G3" t="n">
         <v>0</v>
       </c>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -545,6 +540,7 @@
       <c r="G4" t="n">
         <v>1</v>
       </c>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -572,6 +568,7 @@
       <c r="G5" t="n">
         <v>1</v>
       </c>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -599,6 +596,9 @@
       <c r="G6" t="n">
         <v>1</v>
       </c>
+      <c r="H6" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -626,6 +626,7 @@
       <c r="G7" t="n">
         <v>0</v>
       </c>
+      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -653,6 +654,7 @@
       <c r="G8" t="n">
         <v>0</v>
       </c>
+      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -680,6 +682,7 @@
       <c r="G9" t="n">
         <v>2</v>
       </c>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -707,6 +710,7 @@
       <c r="G10" t="n">
         <v>1</v>
       </c>
+      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -734,6 +738,7 @@
       <c r="G11" t="n">
         <v>2</v>
       </c>
+      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -761,6 +766,7 @@
       <c r="G12" t="n">
         <v>1</v>
       </c>
+      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -788,6 +794,7 @@
       <c r="G13" t="n">
         <v>0</v>
       </c>
+      <c r="H13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: convert counted units to store packs before the cart (#383)
* feat: convert counted units to store packs before the cart (#382)

- optional units_per_pack column: the cart run buys ceil(units needed / units per pack), 0 when nothing is needed, units unchanged when unset
- applied once where the cart run reads the inventory, with one info line per converted item
- item sheet and Add item form carry the field; PUT keeps it when omitted and clears it on null
- "buy" reads units and packs (14 units -> 3 packs) in the Items, Audit and Shop lists
- docs/items.md explains the field; the example sheet gains the column

* test: keep the item sheet e2e within the function-length limit
</commit_message>
<xml_diff>
--- a/data/list.example.xlsx
+++ b/data/list.example.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,43 +413,48 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>super</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>buscador</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>lugar</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>comida</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>cantidad</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>tenemos</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>comprar</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>units_per_pack</t>
         </is>
       </c>
     </row>
@@ -491,6 +484,7 @@
       <c r="G2" t="n">
         <v>1</v>
       </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -518,6 +512,7 @@
       <c r="G3" t="n">
         <v>0</v>
       </c>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -545,6 +540,7 @@
       <c r="G4" t="n">
         <v>1</v>
       </c>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -572,6 +568,7 @@
       <c r="G5" t="n">
         <v>1</v>
       </c>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -599,6 +596,9 @@
       <c r="G6" t="n">
         <v>1</v>
       </c>
+      <c r="H6" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -626,6 +626,7 @@
       <c r="G7" t="n">
         <v>0</v>
       </c>
+      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -653,6 +654,7 @@
       <c r="G8" t="n">
         <v>0</v>
       </c>
+      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -680,6 +682,7 @@
       <c r="G9" t="n">
         <v>2</v>
       </c>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -707,6 +710,7 @@
       <c r="G10" t="n">
         <v>1</v>
       </c>
+      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -734,6 +738,7 @@
       <c r="G11" t="n">
         <v>2</v>
       </c>
+      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -761,6 +766,7 @@
       <c r="G12" t="n">
         <v>1</v>
       </c>
+      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -788,6 +794,7 @@
       <c r="G13" t="n">
         <v>0</v>
       </c>
+      <c r="H13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>